<commit_message>
Auto-export snapshot for 2026-03-17
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -8,7 +8,7 @@
     <sheet state="visible" name="dict" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$54</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$57</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="70">
   <si>
     <t>מאכל</t>
   </si>
@@ -55,22 +55,22 @@
     <t>ולידציה</t>
   </si>
   <si>
-    <t>ביצה</t>
+    <t>יוגור פרו אחוז וחצי</t>
   </si>
   <si>
-    <t>פיתות כוסמין אנג'ל</t>
+    <t>פיתות כוסמין מלא</t>
   </si>
   <si>
     <t>עגלפפון</t>
   </si>
   <si>
-    <t>יוגור פרו אחוז וחצי</t>
+    <t>עוגית חלבון</t>
+  </si>
+  <si>
+    <t>ביצה</t>
   </si>
   <si>
     <t>שמן זית</t>
-  </si>
-  <si>
-    <t>פרגית</t>
   </si>
   <si>
     <t>בצל</t>
@@ -88,31 +88,34 @@
     <t>אורז</t>
   </si>
   <si>
-    <t>קוואקר</t>
-  </si>
-  <si>
-    <t>קוטג 5</t>
-  </si>
-  <si>
-    <t>חטיף חלבון פיסטוק</t>
+    <t>גרנולה לא מתוקה</t>
   </si>
   <si>
     <t>דבש</t>
   </si>
   <si>
-    <t>עוגית חלבון</t>
+    <t>בננה</t>
   </si>
   <si>
-    <t>פסטה אוסם</t>
+    <t>יוגורט פרו מתוק</t>
   </si>
   <si>
-    <t>_</t>
+    <t>חטיף חלבון פיסטוק</t>
   </si>
   <si>
     <t>יוגורט פרו זירו</t>
   </si>
   <si>
     <t>פסטרמה</t>
+  </si>
+  <si>
+    <t>אצבעות מוצרלה</t>
+  </si>
+  <si>
+    <t>פיתות כוסמין אנג'ל</t>
+  </si>
+  <si>
+    <t>_</t>
   </si>
   <si>
     <t>אוכל</t>
@@ -130,25 +133,16 @@
     <t>אולין בוטנים קרמל</t>
   </si>
   <si>
-    <t>אצבעות מוצרלה</t>
-  </si>
-  <si>
     <t>אצבעות עמק</t>
   </si>
   <si>
     <t>בטטה</t>
   </si>
   <si>
-    <t>בננה</t>
-  </si>
-  <si>
     <t>גזר</t>
   </si>
   <si>
     <t>גמבה</t>
-  </si>
-  <si>
-    <t>גרנולה לא מתוקה</t>
   </si>
   <si>
     <t>זית</t>
@@ -170,9 +164,6 @@
   </si>
   <si>
     <t>טופו קשה</t>
-  </si>
-  <si>
-    <t>יוגורט פרו מתוק</t>
   </si>
   <si>
     <t>כדור תמרים</t>
@@ -208,7 +199,16 @@
     <t>פיתות כוסמין לבן</t>
   </si>
   <si>
-    <t>פיתות כוסמין מלא</t>
+    <t>פסטה אוסם</t>
+  </si>
+  <si>
+    <t>פרגית</t>
+  </si>
+  <si>
+    <t>קוואקר</t>
+  </si>
+  <si>
+    <t>קוטג 5</t>
   </si>
   <si>
     <t>קטניות</t>
@@ -221,6 +221,15 @@
   </si>
   <si>
     <t>תערובת ירוקים</t>
+  </si>
+  <si>
+    <t>ריבר בוט בינוני</t>
+  </si>
+  <si>
+    <t>חטיף טודיי</t>
+  </si>
+  <si>
+    <t>פיתות כוסמין לוי</t>
   </si>
 </sst>
 </file>
@@ -553,43 +562,43 @@
         <v>11</v>
       </c>
       <c r="B2" s="3">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="C2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 3, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>1</v>
+        <v>6.8</v>
       </c>
       <c r="D2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 4, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 5, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="F2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 6, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>194</v>
+        <v>140</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>372.61</v>
+        <v>339.35</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>224.07</v>
+        <v>196.9</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>82.09</v>
+        <v>54.87</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3108.2</v>
+        <v>2649.59</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>3125.53</v>
+        <v>2638.83</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -601,19 +610,19 @@
       </c>
       <c r="C3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 3, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>37.4</v>
       </c>
       <c r="D3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 4, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>8.8</v>
       </c>
       <c r="E3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 5, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>2.09</v>
       </c>
       <c r="F3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 6, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -621,11 +630,11 @@
         <v>13</v>
       </c>
       <c r="B4" s="3">
-        <v>180.0</v>
+        <v>200.0</v>
       </c>
       <c r="C4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 3, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="D4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 4, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
@@ -637,7 +646,7 @@
       </c>
       <c r="F4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 6, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -645,23 +654,23 @@
         <v>14</v>
       </c>
       <c r="B5" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 3, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>6.8</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 4, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 5, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 6, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>140</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -669,31 +678,31 @@
         <v>15</v>
       </c>
       <c r="B6" s="3">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="C6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 3, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 4, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 5, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>4.6</v>
+        <v>13</v>
       </c>
       <c r="F6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 6, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>41.5</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="3">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="C7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 3, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
@@ -705,11 +714,11 @@
       </c>
       <c r="E7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 5, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>9.2</v>
+        <v>6.44</v>
       </c>
       <c r="F7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 6, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>83</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -717,7 +726,7 @@
         <v>16</v>
       </c>
       <c r="B8" s="3">
-        <v>100.0</v>
+        <v>5.0</v>
       </c>
       <c r="C8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 3, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
@@ -725,15 +734,15 @@
       </c>
       <c r="D8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 4, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 5, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>9</v>
+        <v>4.6</v>
       </c>
       <c r="F8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 6, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>175</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -741,23 +750,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>150.0</v>
+        <v>180.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>14.01</v>
+        <v>16.812</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>1.65</v>
+        <v>1.98</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>60</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -765,23 +774,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="3">
-        <v>200.0</v>
+        <v>390.0</v>
       </c>
       <c r="C10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>3.4</v>
+        <v>6.63</v>
       </c>
       <c r="E10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>172</v>
+        <v>335.4</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -789,7 +798,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>170.0</v>
+        <v>193.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -797,15 +806,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>42.5</v>
+        <v>48.25</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4.25</v>
+        <v>4.825</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>204</v>
+        <v>231.6</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -813,23 +822,23 @@
         <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="C12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 3, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>35.2</v>
+        <v>31.68</v>
       </c>
       <c r="D12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 4, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="E12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 5, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>1.3</v>
+        <v>1.17</v>
       </c>
       <c r="F12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 6, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>176.5</v>
+        <v>158.85</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -837,15 +846,15 @@
         <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="C13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 3, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>39</v>
+        <v>35.1</v>
       </c>
       <c r="D13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 4, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>4.4</v>
+        <v>3.96</v>
       </c>
       <c r="E13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 5, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
@@ -853,7 +862,7 @@
       </c>
       <c r="F13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 6, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>175</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -861,23 +870,23 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>50.0</v>
+        <v>30.0</v>
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>34.5</v>
+        <v>15.54</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>5.5</v>
+        <v>4.41</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>4.35</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>187</v>
+        <v>115.2</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -886,11 +895,11 @@
         <v>23</v>
       </c>
       <c r="B15" s="3">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="C15" s="4">
         <f>VLOOKUP($A15, dict!$A:$F, 3, false) * $B15 / VLOOKUP($A15, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D15" s="4">
         <f>VLOOKUP($A15, dict!$A:$F, 4, false) * $B15 / VLOOKUP($A15, dict!$A:$F, 2, false)</f>
@@ -902,72 +911,74 @@
       </c>
       <c r="F15" s="4">
         <f>VLOOKUP($A15, dict!$A:$F, 6, false) * $B15 / VLOOKUP($A15, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G15" s="4"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" s="3">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="C16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 3, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>21.7</v>
+        <v>4</v>
       </c>
       <c r="D16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 4, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 5, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 6, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>212</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G16" s="4"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3">
-        <v>10.0</v>
+        <v>127.0</v>
       </c>
       <c r="C17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 3, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>8</v>
+        <v>29.718</v>
       </c>
       <c r="D17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 4, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>1.27</v>
       </c>
       <c r="E17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 5, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>0.635</v>
       </c>
       <c r="F17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 6, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>32</v>
-      </c>
+        <v>116.84</v>
+      </c>
+      <c r="G17" s="4"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="C18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 3, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>11.2</v>
       </c>
       <c r="D18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 4, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 5, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
@@ -975,7 +986,7 @@
       </c>
       <c r="F18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 6, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
@@ -983,23 +994,23 @@
         <v>26</v>
       </c>
       <c r="B19" s="3">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="C19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 3, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>11.5</v>
+        <v>0</v>
       </c>
       <c r="D19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 4, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="E19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 5, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>4.45</v>
+        <v>0</v>
       </c>
       <c r="F19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 6, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -1007,11 +1018,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="5">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
       <c r="C20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 3, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="D20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 4, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
@@ -1023,63 +1034,63 @@
       </c>
       <c r="F20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 6, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B21" s="5">
-        <v>180.0</v>
+        <v>1.0</v>
       </c>
       <c r="C21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 3, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="D21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 4, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="E21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 5, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="F21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 6, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>216</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" s="5">
-        <v>100.0</v>
+        <v>5.0</v>
       </c>
       <c r="C22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 3, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>71</v>
+        <v>5.5</v>
       </c>
       <c r="D22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 4, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 5, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="F22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 6, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>349</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B23" s="5">
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="C23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 3, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
@@ -1087,15 +1098,15 @@
       </c>
       <c r="D23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 4, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>10.4</v>
       </c>
       <c r="E23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 5, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>9.2</v>
+        <v>8.6</v>
       </c>
       <c r="F23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 6, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>83</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -1107,24 +1118,43 @@
       </c>
       <c r="C24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 3, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>37.4</v>
       </c>
       <c r="D24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 4, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>8.8</v>
       </c>
       <c r="E24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 5, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>2.09</v>
       </c>
       <c r="F24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 6, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="3" t="s">
-        <v>28</v>
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="5">
+        <v>10.0</v>
+      </c>
+      <c r="C25" s="4">
+        <f>VLOOKUP($A25, dict!$A:$F, 3, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
+        <v>8</v>
+      </c>
+      <c r="D25" s="4">
+        <f>VLOOKUP($A25, dict!$A:$F, 4, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <f>VLOOKUP($A25, dict!$A:$F, 5, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="4">
+        <f>VLOOKUP($A25, dict!$A:$F, 6, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
+        <v>32</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -4116,7 +4146,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B2" s="3">
         <v>110.0</v>
@@ -4160,7 +4190,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B3" s="3">
         <v>1.0</v>
@@ -4184,7 +4214,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3">
         <v>5.0</v>
@@ -4232,7 +4262,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
@@ -4256,7 +4286,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -7260,10 +7290,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7278,12 +7308,12 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B2" s="4">
         <v>1.0</v>
@@ -7303,7 +7333,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="4">
         <v>1.0</v>
@@ -7321,13 +7351,13 @@
         <v>110.0</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G54" si="1">4*C3 + 4*D3 + 9*E3</f>
+        <f t="shared" ref="G3:G57" si="1">4*C3 + 4*D3 + 9*E3</f>
         <v>113</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="5">
         <v>1.0</v>
@@ -7375,7 +7405,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4">
         <v>1.0</v>
@@ -7447,7 +7477,7 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B9" s="4">
         <v>1.0</v>
@@ -7471,7 +7501,7 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B10" s="4">
         <v>100.0</v>
@@ -7519,7 +7549,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="5">
         <v>100.0</v>
@@ -7543,7 +7573,7 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="4">
         <v>100.0</v>
@@ -7567,7 +7597,7 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B14" s="4">
         <v>100.0</v>
@@ -7591,7 +7621,7 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" s="5">
         <v>100.0</v>
@@ -7615,7 +7645,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B16" s="5">
         <v>4.0</v>
@@ -7663,7 +7693,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B18" s="5">
         <v>1.0</v>
@@ -7687,7 +7717,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B19" s="5">
         <v>1.0</v>
@@ -7711,7 +7741,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B20" s="5">
         <v>1.0</v>
@@ -7735,7 +7765,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B21" s="4">
         <v>1.0</v>
@@ -7759,7 +7789,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B22" s="4">
         <v>100.0</v>
@@ -7783,7 +7813,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B23" s="5">
         <v>100.0</v>
@@ -7807,7 +7837,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B24" s="4">
         <v>100.0</v>
@@ -7831,7 +7861,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B25" s="4">
         <v>1.0</v>
@@ -7855,7 +7885,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B26" s="4">
         <v>1.0</v>
@@ -7879,7 +7909,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="B27" s="4">
         <v>1.0</v>
@@ -7903,7 +7933,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B28" s="4">
         <v>1.0</v>
@@ -7951,7 +7981,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B30" s="5">
         <v>100.0</v>
@@ -7975,7 +8005,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B31" s="5">
         <v>100.0</v>
@@ -7999,7 +8029,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B32" s="5">
         <v>1.0</v>
@@ -8023,7 +8053,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B33" s="4">
         <v>100.0</v>
@@ -8047,7 +8077,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B34" s="4">
         <v>100.0</v>
@@ -8071,7 +8101,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B35" s="5">
         <v>100.0</v>
@@ -8095,7 +8125,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B36" s="4">
         <v>100.0</v>
@@ -8143,7 +8173,7 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="7" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B38" s="5">
         <v>1.0</v>
@@ -8167,7 +8197,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B39" s="4">
         <v>100.0</v>
@@ -8191,7 +8221,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B40" s="5">
         <v>100.0</v>
@@ -8215,7 +8245,7 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B41" s="4">
         <v>100.0</v>
@@ -8239,7 +8269,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B42" s="5">
         <v>100.0</v>
@@ -8263,7 +8293,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="B43" s="3">
         <v>100.0</v>
@@ -8287,7 +8317,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="7" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="B44" s="5">
         <v>100.0</v>
@@ -8311,7 +8341,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B45" s="4">
         <v>1.0</v>
@@ -8335,7 +8365,7 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="B46" s="4">
         <v>100.0</v>
@@ -8359,7 +8389,7 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="B47" s="4">
         <v>100.0</v>
@@ -8383,7 +8413,7 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="7" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="B48" s="5">
         <v>100.0</v>
@@ -8479,7 +8509,7 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B52" s="4">
         <v>100.0</v>
@@ -8549,9 +8579,78 @@
         <v>87.7</v>
       </c>
     </row>
-    <row r="55" ht="15.75" customHeight="1"/>
-    <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="A55" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="C55" s="5">
+        <v>60.0</v>
+      </c>
+      <c r="D55" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="E55" s="5">
+        <v>10.0</v>
+      </c>
+      <c r="F55" s="5">
+        <v>455.0</v>
+      </c>
+      <c r="G55" s="4">
+        <f t="shared" si="1"/>
+        <v>410</v>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B56" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="C56" s="5">
+        <v>16.0</v>
+      </c>
+      <c r="D56" s="5">
+        <v>18.0</v>
+      </c>
+      <c r="E56" s="5">
+        <v>3.2</v>
+      </c>
+      <c r="F56" s="5">
+        <v>185.0</v>
+      </c>
+      <c r="G56" s="4">
+        <f t="shared" si="1"/>
+        <v>164.8</v>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B57" s="5">
+        <v>100.0</v>
+      </c>
+      <c r="C57" s="5">
+        <v>29.8</v>
+      </c>
+      <c r="D57" s="5">
+        <v>12.4</v>
+      </c>
+      <c r="E57" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="F57" s="5">
+        <v>216.0</v>
+      </c>
+      <c r="G57" s="4">
+        <f t="shared" si="1"/>
+        <v>176.9</v>
+      </c>
+    </row>
     <row r="58" ht="15.75" customHeight="1"/>
     <row r="59" ht="15.75" customHeight="1"/>
     <row r="60" ht="15.75" customHeight="1"/>
@@ -9497,9 +9596,9 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$G$54">
-    <sortState ref="A1:G54">
-      <sortCondition ref="A1:A54"/>
+  <autoFilter ref="$A$1:$G$57">
+    <sortState ref="A1:G57">
+      <sortCondition ref="A1:A57"/>
     </sortState>
   </autoFilter>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-19
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -8,7 +8,7 @@
     <sheet state="visible" name="dict" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$57</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="72">
   <si>
     <t>מאכל</t>
   </si>
@@ -55,7 +55,7 @@
     <t>ולידציה</t>
   </si>
   <si>
-    <t>יוגור פרו אחוז וחצי</t>
+    <t>יוגורט פרו זירו</t>
   </si>
   <si>
     <t>פיתות כוסמין מלא</t>
@@ -88,7 +88,7 @@
     <t>אורז</t>
   </si>
   <si>
-    <t>גרנולה לא מתוקה</t>
+    <t xml:space="preserve">גרנולה שוקולד </t>
   </si>
   <si>
     <t>דבש</t>
@@ -103,16 +103,16 @@
     <t>חטיף חלבון פיסטוק</t>
   </si>
   <si>
-    <t>יוגורט פרו זירו</t>
-  </si>
-  <si>
-    <t>פסטרמה</t>
+    <t>גיינר</t>
   </si>
   <si>
     <t>אצבעות מוצרלה</t>
   </si>
   <si>
     <t>פיתות כוסמין אנג'ל</t>
+  </si>
+  <si>
+    <t>פסטרמה</t>
   </si>
   <si>
     <t>_</t>
@@ -145,6 +145,9 @@
     <t>גמבה</t>
   </si>
   <si>
+    <t>גרנולה לא מתוקה</t>
+  </si>
+  <si>
     <t>זית</t>
   </si>
   <si>
@@ -164,6 +167,9 @@
   </si>
   <si>
     <t>טופו קשה</t>
+  </si>
+  <si>
+    <t>יוגור פרו אחוז וחצי</t>
   </si>
   <si>
     <t>כדור תמרים</t>
@@ -566,7 +572,7 @@
       </c>
       <c r="C2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 3, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="D2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 4, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
@@ -574,31 +580,31 @@
       </c>
       <c r="E2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 5, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 6, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>339.35</v>
+        <v>364.6288</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>196.9</v>
+        <v>178.664</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>54.87</v>
+        <v>45.293</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>2649.59</v>
+        <v>2613.85</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2638.83</v>
+        <v>2580.8082</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -725,9 +731,7 @@
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3">
-        <v>5.0</v>
-      </c>
+      <c r="B8" s="3"/>
       <c r="C8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 3, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
         <v>0</v>
@@ -738,11 +742,11 @@
       </c>
       <c r="E8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 5, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="F8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 6, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>41.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -750,23 +754,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>180.0</v>
+        <v>162.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>16.812</v>
+        <v>15.1308</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>1.98</v>
+        <v>1.782</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.18</v>
+        <v>0.162</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>72</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -774,23 +778,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="3">
-        <v>390.0</v>
+        <v>356.0</v>
       </c>
       <c r="C10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>78</v>
+        <v>71.2</v>
       </c>
       <c r="D10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>6.63</v>
+        <v>6.052</v>
       </c>
       <c r="E10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.39</v>
+        <v>0.356</v>
       </c>
       <c r="F10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>335.4</v>
+        <v>306.16</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -798,7 +802,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>193.0</v>
+        <v>170.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -806,15 +810,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>48.25</v>
+        <v>42.5</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4.825</v>
+        <v>4.25</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>231.6</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -874,19 +878,19 @@
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>15.54</v>
+        <v>18.9</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4.41</v>
+        <v>2.7</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4.35</v>
+        <v>4.5</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>115.2</v>
+        <v>130.5</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -1039,7 +1043,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B21" s="5">
         <v>1.0</v>
@@ -1063,31 +1067,31 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="5">
-        <v>5.0</v>
+        <v>50.0</v>
       </c>
       <c r="C22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 3, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>5.5</v>
+        <v>36</v>
       </c>
       <c r="D22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 4, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 5, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="F22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 6, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>120</v>
+        <v>198.5</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="5">
         <v>2.0</v>
@@ -4146,7 +4150,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" s="3">
         <v>110.0</v>
@@ -4190,7 +4194,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3">
         <v>1.0</v>
@@ -4262,7 +4266,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
@@ -7351,7 +7355,7 @@
         <v>110.0</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G57" si="1">4*C3 + 4*D3 + 9*E3</f>
+        <f t="shared" ref="G3:G59" si="1">4*C3 + 4*D3 + 9*E3</f>
         <v>113</v>
       </c>
     </row>
@@ -7405,7 +7409,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="4">
         <v>1.0</v>
@@ -7597,7 +7601,7 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4">
         <v>100.0</v>
@@ -7645,7 +7649,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="5">
         <v>4.0</v>
@@ -7693,7 +7697,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" s="5">
         <v>1.0</v>
@@ -7741,7 +7745,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" s="5">
         <v>1.0</v>
@@ -7765,7 +7769,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" s="4">
         <v>1.0</v>
@@ -7789,7 +7793,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" s="4">
         <v>100.0</v>
@@ -7813,7 +7817,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B23" s="5">
         <v>100.0</v>
@@ -7837,7 +7841,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="4">
         <v>100.0</v>
@@ -7861,7 +7865,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4">
         <v>1.0</v>
@@ -7885,7 +7889,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B26" s="4">
         <v>1.0</v>
@@ -7933,7 +7937,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4">
         <v>1.0</v>
@@ -7981,7 +7985,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B30" s="5">
         <v>100.0</v>
@@ -8005,7 +8009,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B31" s="5">
         <v>100.0</v>
@@ -8029,7 +8033,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B32" s="5">
         <v>1.0</v>
@@ -8053,7 +8057,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B33" s="4">
         <v>100.0</v>
@@ -8077,7 +8081,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B34" s="4">
         <v>100.0</v>
@@ -8101,7 +8105,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B35" s="5">
         <v>100.0</v>
@@ -8125,7 +8129,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B36" s="4">
         <v>100.0</v>
@@ -8197,7 +8201,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B39" s="4">
         <v>100.0</v>
@@ -8221,7 +8225,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B40" s="5">
         <v>100.0</v>
@@ -8245,7 +8249,7 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B41" s="4">
         <v>100.0</v>
@@ -8269,7 +8273,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B42" s="5">
         <v>100.0</v>
@@ -8317,7 +8321,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B44" s="5">
         <v>100.0</v>
@@ -8341,7 +8345,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4">
         <v>1.0</v>
@@ -8365,7 +8369,7 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B46" s="4">
         <v>100.0</v>
@@ -8389,7 +8393,7 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B47" s="4">
         <v>100.0</v>
@@ -8413,7 +8417,7 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B48" s="5">
         <v>100.0</v>
@@ -8437,7 +8441,7 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B49" s="4">
         <v>100.0</v>
@@ -8461,7 +8465,7 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B50" s="5">
         <v>100.0</v>
@@ -8485,7 +8489,7 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B51" s="4">
         <v>100.0</v>
@@ -8533,7 +8537,7 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B53" s="4">
         <v>100.0</v>
@@ -8581,7 +8585,7 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B55" s="5">
         <v>1.0</v>
@@ -8605,7 +8609,7 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B56" s="5">
         <v>1.0</v>
@@ -8629,7 +8633,7 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B57" s="5">
         <v>100.0</v>
@@ -8651,8 +8655,54 @@
         <v>176.9</v>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B58" s="5">
+        <v>100.0</v>
+      </c>
+      <c r="C58" s="5">
+        <v>72.0</v>
+      </c>
+      <c r="D58" s="5">
+        <v>16.0</v>
+      </c>
+      <c r="E58" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="F58" s="5">
+        <v>397.0</v>
+      </c>
+      <c r="G58" s="4">
+        <f t="shared" si="1"/>
+        <v>388</v>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B59" s="5">
+        <v>100.0</v>
+      </c>
+      <c r="C59" s="5">
+        <v>63.0</v>
+      </c>
+      <c r="D59" s="5">
+        <v>9.0</v>
+      </c>
+      <c r="E59" s="5">
+        <v>15.0</v>
+      </c>
+      <c r="F59" s="5">
+        <v>435.0</v>
+      </c>
+      <c r="G59" s="4">
+        <f t="shared" si="1"/>
+        <v>423</v>
+      </c>
+    </row>
     <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -9596,9 +9646,9 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$G$57">
-    <sortState ref="A1:G57">
-      <sortCondition ref="A1:A57"/>
+  <autoFilter ref="$A$1:$G$59">
+    <sortState ref="A1:G59">
+      <sortCondition ref="A1:A59"/>
     </sortState>
   </autoFilter>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-20
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -109,6 +109,9 @@
     <t>אצבעות מוצרלה</t>
   </si>
   <si>
+    <t>פיתות כוסמין מלא</t>
+  </si>
+  <si>
     <t>פסטרמה</t>
   </si>
   <si>
@@ -200,9 +203,6 @@
   </si>
   <si>
     <t>פיתות כוסמין לבן</t>
-  </si>
-  <si>
-    <t>פיתות כוסמין מלא</t>
   </si>
   <si>
     <t>פסטה אוסם</t>
@@ -588,23 +588,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>372.4748</v>
+        <v>335.9144</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>182.774</v>
+        <v>194.492</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>46.198</v>
+        <v>65.974</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>2668.43</v>
+        <v>2735.85</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2636.7772</v>
+        <v>2715.3916</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -660,23 +660,23 @@
         <v>14</v>
       </c>
       <c r="B5" s="3">
-        <v>0.0</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 3, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="D5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 4, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="E5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 5, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>4.45</v>
       </c>
       <c r="F5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 6, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -708,7 +708,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="3">
-        <v>7.0</v>
+        <v>10.0</v>
       </c>
       <c r="C7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 3, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
@@ -720,11 +720,11 @@
       </c>
       <c r="E7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 5, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>6.44</v>
+        <v>9.2</v>
       </c>
       <c r="F7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 6, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>58.1</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -732,7 +732,7 @@
         <v>16</v>
       </c>
       <c r="B8" s="3">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="C8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 3, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
@@ -744,11 +744,11 @@
       </c>
       <c r="E8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 5, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="F8" s="4">
         <f>VLOOKUP($A8, dict!$A:$F, 6, false) * $B8 / VLOOKUP($A8, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -756,23 +756,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>162.0</v>
+        <v>156.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>15.1308</v>
+        <v>14.5704</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>1.782</v>
+        <v>1.716</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.162</v>
+        <v>0.156</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>64.8</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -780,23 +780,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="3">
-        <v>356.0</v>
+        <v>288.0</v>
       </c>
       <c r="C10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>71.2</v>
+        <v>57.6</v>
       </c>
       <c r="D10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>6.052</v>
+        <v>4.896</v>
       </c>
       <c r="E10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.356</v>
+        <v>0.288</v>
       </c>
       <c r="F10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>306.16</v>
+        <v>247.68</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -926,11 +926,11 @@
         <v>23</v>
       </c>
       <c r="B16" s="3">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="C16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 3, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 4, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
@@ -942,7 +942,7 @@
       </c>
       <c r="F16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 6, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -1024,11 +1024,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="5">
-        <v>100.0</v>
+        <v>0.0</v>
       </c>
       <c r="C20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 3, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 4, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="F20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 6, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -1072,23 +1072,23 @@
         <v>27</v>
       </c>
       <c r="B22" s="5">
-        <v>50.0</v>
+        <v>40.0</v>
       </c>
       <c r="C22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 3, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>36</v>
+        <v>28.8</v>
       </c>
       <c r="D22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 4, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>8</v>
+        <v>6.4</v>
       </c>
       <c r="E22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 5, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="F22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 6, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>198.5</v>
+        <v>158.8</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -1096,7 +1096,7 @@
         <v>28</v>
       </c>
       <c r="B23" s="5">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 3, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
@@ -1104,51 +1104,49 @@
       </c>
       <c r="D23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 4, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>10.4</v>
+        <v>20.8</v>
       </c>
       <c r="E23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 5, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>8.6</v>
+        <v>17.2</v>
       </c>
       <c r="F23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 6, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>118</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B24" s="5">
-        <v>110.0</v>
+        <v>90.0</v>
       </c>
       <c r="C24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 3, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>30.6</v>
       </c>
       <c r="D24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 4, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>7.2</v>
       </c>
       <c r="E24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 5, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>1.71</v>
       </c>
       <c r="F24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 6, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>178.2</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="5">
-        <v>10.0</v>
-      </c>
+      <c r="B25" s="5"/>
       <c r="C25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 3, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 4, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
@@ -1160,7 +1158,7 @@
       </c>
       <c r="F25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 6, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -4268,7 +4266,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
@@ -4292,7 +4290,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -7296,10 +7294,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7314,12 +7312,12 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="4">
         <v>1.0</v>
@@ -7339,7 +7337,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="4">
         <v>1.0</v>
@@ -7363,7 +7361,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="5">
         <v>1.0</v>
@@ -7435,7 +7433,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4">
         <v>1.0</v>
@@ -7459,7 +7457,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="5">
         <v>100.0</v>
@@ -7555,7 +7553,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="5">
         <v>100.0</v>
@@ -7579,7 +7577,7 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" s="4">
         <v>100.0</v>
@@ -7603,7 +7601,7 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4">
         <v>100.0</v>
@@ -7651,7 +7649,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="5">
         <v>4.0</v>
@@ -7699,7 +7697,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" s="5">
         <v>1.0</v>
@@ -7747,7 +7745,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" s="5">
         <v>1.0</v>
@@ -7771,7 +7769,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" s="4">
         <v>1.0</v>
@@ -7795,7 +7793,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" s="4">
         <v>100.0</v>
@@ -7819,7 +7817,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B23" s="5">
         <v>100.0</v>
@@ -7843,7 +7841,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="4">
         <v>100.0</v>
@@ -7867,7 +7865,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4">
         <v>1.0</v>
@@ -7939,7 +7937,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4">
         <v>1.0</v>
@@ -7987,7 +7985,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="5">
         <v>100.0</v>
@@ -8011,7 +8009,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="5">
         <v>100.0</v>
@@ -8035,7 +8033,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B32" s="5">
         <v>1.0</v>
@@ -8059,7 +8057,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B33" s="4">
         <v>100.0</v>
@@ -8083,7 +8081,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B34" s="4">
         <v>100.0</v>
@@ -8107,7 +8105,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B35" s="5">
         <v>100.0</v>
@@ -8131,7 +8129,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B36" s="4">
         <v>100.0</v>
@@ -8203,7 +8201,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B39" s="4">
         <v>100.0</v>
@@ -8227,7 +8225,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B40" s="5">
         <v>100.0</v>
@@ -8275,7 +8273,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B42" s="5">
         <v>100.0</v>
@@ -8299,7 +8297,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="B43" s="3">
         <v>100.0</v>
@@ -8347,7 +8345,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4">
         <v>1.0</v>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-22
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -588,23 +588,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>335.9144</v>
+        <v>411.624</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>194.492</v>
+        <v>193.232</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>65.974</v>
+        <v>54.706</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>2735.85</v>
+        <v>2956.33</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2715.3916</v>
+        <v>2911.778</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -660,23 +660,23 @@
         <v>14</v>
       </c>
       <c r="B5" s="3">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="C5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 3, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>11.5</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 4, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="E5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 5, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>4.45</v>
+        <v>0</v>
       </c>
       <c r="F5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 6, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -708,7 +708,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="3">
-        <v>10.0</v>
+        <v>7.0</v>
       </c>
       <c r="C7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 3, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
@@ -720,11 +720,11 @@
       </c>
       <c r="E7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 5, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>9.2</v>
+        <v>6.44</v>
       </c>
       <c r="F7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 6, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>83</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -756,23 +756,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>156.0</v>
+        <v>200.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>14.5704</v>
+        <v>18.68</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>1.716</v>
+        <v>2.2</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.156</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>62.4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -780,23 +780,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="3">
-        <v>288.0</v>
+        <v>256.0</v>
       </c>
       <c r="C10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>57.6</v>
+        <v>51.2</v>
       </c>
       <c r="D10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>4.896</v>
+        <v>4.352</v>
       </c>
       <c r="E10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.288</v>
+        <v>0.256</v>
       </c>
       <c r="F10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>247.68</v>
+        <v>220.16</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -804,7 +804,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>170.0</v>
+        <v>160.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -812,15 +812,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>42.5</v>
+        <v>40</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -1024,11 +1024,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="5">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
       <c r="C20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 3, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="D20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 4, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="F20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 6, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -1072,23 +1072,23 @@
         <v>27</v>
       </c>
       <c r="B22" s="5">
-        <v>40.0</v>
+        <v>150.0</v>
       </c>
       <c r="C22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 3, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>28.8</v>
+        <v>108</v>
       </c>
       <c r="D22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 4, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>6.4</v>
+        <v>24</v>
       </c>
       <c r="E22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 5, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>1.6</v>
+        <v>6</v>
       </c>
       <c r="F22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 6, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>158.8</v>
+        <v>595.5</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -1096,7 +1096,7 @@
         <v>28</v>
       </c>
       <c r="B23" s="5">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="C23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 3, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
@@ -1104,15 +1104,15 @@
       </c>
       <c r="D23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 4, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>20.8</v>
+        <v>10.4</v>
       </c>
       <c r="E23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 5, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>17.2</v>
+        <v>8.6</v>
       </c>
       <c r="F23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 6, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>236</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -1120,30 +1120,32 @@
         <v>29</v>
       </c>
       <c r="B24" s="5">
-        <v>90.0</v>
+        <v>110.0</v>
       </c>
       <c r="C24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 3, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>30.6</v>
+        <v>37.4</v>
       </c>
       <c r="D24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 4, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>7.2</v>
+        <v>8.8</v>
       </c>
       <c r="E24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 5, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>1.71</v>
+        <v>2.09</v>
       </c>
       <c r="F24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 6, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>178.2</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="B25" s="5">
+        <v>0.0</v>
+      </c>
       <c r="C25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 3, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
         <v>0</v>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-23
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -588,23 +588,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>421.624</v>
+        <v>384.9488</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>203.232</v>
+        <v>212.072</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>65.306</v>
+        <v>63.802</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3120.83</v>
+        <v>3014.65</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>3087.178</v>
+        <v>2962.3012</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -756,23 +756,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>200.0</v>
+        <v>232.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>18.68</v>
+        <v>21.6688</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>2.2</v>
+        <v>2.552</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.2</v>
+        <v>0.232</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>80</v>
+        <v>92.8</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -780,23 +780,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="3">
-        <v>256.0</v>
+        <v>200.0</v>
       </c>
       <c r="C10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>51.2</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>4.352</v>
+        <v>3.4</v>
       </c>
       <c r="E10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.256</v>
+        <v>0.2</v>
       </c>
       <c r="F10" s="4">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>220.16</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -804,7 +804,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>160.0</v>
+        <v>200.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -812,15 +812,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>192</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -951,23 +951,23 @@
         <v>24</v>
       </c>
       <c r="B17" s="3">
-        <v>96.0</v>
+        <v>0.0</v>
       </c>
       <c r="C17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 3, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>22.464</v>
+        <v>0</v>
       </c>
       <c r="D17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 4, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>0.96</v>
+        <v>0</v>
       </c>
       <c r="E17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 5, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="F17" s="4">
         <f>VLOOKUP($A17, dict!$A:$F, 6, false) * $B17 / VLOOKUP($A17, dict!$A:$F, 2, false)</f>
-        <v>88.32</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4"/>
     </row>
@@ -1072,23 +1072,23 @@
         <v>26</v>
       </c>
       <c r="B22" s="5">
-        <v>120.0</v>
+        <v>150.0</v>
       </c>
       <c r="C22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 3, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>86.4</v>
+        <v>108</v>
       </c>
       <c r="D22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 4, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>19.2</v>
+        <v>24</v>
       </c>
       <c r="E22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 5, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="F22" s="4">
         <f>VLOOKUP($A22, dict!$A:$F, 6, false) * $B22 / VLOOKUP($A22, dict!$A:$F, 2, false)</f>
-        <v>476.4</v>
+        <v>595.5</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -1144,23 +1144,23 @@
         <v>29</v>
       </c>
       <c r="B25" s="5">
-        <v>40.0</v>
+        <v>0.0</v>
       </c>
       <c r="C25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 3, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>27.6</v>
+        <v>0</v>
       </c>
       <c r="D25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 4, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="E25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 5, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="F25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 6, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>149.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-27
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="72">
   <si>
     <t>מאכל</t>
   </si>
@@ -106,10 +106,13 @@
     <t>אצבעות מוצרלה</t>
   </si>
   <si>
-    <t>פיתות כוסמין מלא</t>
+    <t>קוואקר</t>
   </si>
   <si>
-    <t>קוואקר</t>
+    <t>נודלס אורז</t>
+  </si>
+  <si>
+    <t>טופו קשה</t>
   </si>
   <si>
     <t>פסטרמה</t>
@@ -169,9 +172,6 @@
     <t>טונה</t>
   </si>
   <si>
-    <t>טופו קשה</t>
-  </si>
-  <si>
     <t>יוגור פרו אחוז וחצי</t>
   </si>
   <si>
@@ -185,9 +185,6 @@
   </si>
   <si>
     <t>מנה חמה בקר</t>
-  </si>
-  <si>
-    <t>נודלס אורז</t>
   </si>
   <si>
     <t>נודלס חיטה</t>
@@ -206,6 +203,9 @@
   </si>
   <si>
     <t>פיתות כוסמין לבן</t>
+  </si>
+  <si>
+    <t>פיתות כוסמין מלא</t>
   </si>
   <si>
     <t>פסטה אוסם</t>
@@ -595,23 +595,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>387.7014</v>
+        <v>412.113</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>211.863</v>
+        <v>204.365</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>63.717</v>
+        <v>60.225</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3023.26</v>
+        <v>3058.3</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2971.7106</v>
+        <v>3007.937</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -763,23 +763,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>221.0</v>
+        <v>195.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>20.6414</v>
+        <v>18.213</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>2.431</v>
+        <v>2.145</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.221</v>
+        <v>0.195</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>88.4</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -787,23 +787,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="5">
-        <v>256.0</v>
+        <v>300.0</v>
       </c>
       <c r="C10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>51.2</v>
+        <v>60</v>
       </c>
       <c r="D10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>4.352</v>
+        <v>5.1</v>
       </c>
       <c r="E10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.256</v>
+        <v>0.3</v>
       </c>
       <c r="F10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>220.16</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -811,7 +811,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>200.0</v>
+        <v>170.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -819,15 +819,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>50</v>
+        <v>42.5</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>5</v>
+        <v>4.25</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>240</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -835,23 +835,23 @@
         <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>40.0</v>
+        <v>50.0</v>
       </c>
       <c r="C12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 3, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>28.16</v>
+        <v>35.2</v>
       </c>
       <c r="D12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 4, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="E12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 5, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>1.04</v>
+        <v>1.3</v>
       </c>
       <c r="F12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 6, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>141.2</v>
+        <v>176.5</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -859,15 +859,15 @@
         <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>40.0</v>
+        <v>50.0</v>
       </c>
       <c r="C13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 3, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>31.2</v>
+        <v>39</v>
       </c>
       <c r="D13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 4, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>3.52</v>
+        <v>4.4</v>
       </c>
       <c r="E13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 5, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
@@ -875,7 +875,7 @@
       </c>
       <c r="F13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 6, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>140</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -883,23 +883,23 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>40.0</v>
+        <v>50.0</v>
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>25.2</v>
+        <v>31.5</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>174</v>
+        <v>217.5</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -1007,11 +1007,11 @@
         <v>23</v>
       </c>
       <c r="B19" s="3">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="C19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 3, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 4, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="F19" s="4">
         <f>VLOOKUP($A19, dict!$A:$F, 6, false) * $B19 / VLOOKUP($A19, dict!$A:$F, 2, false)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -1031,11 +1031,11 @@
         <v>13</v>
       </c>
       <c r="B20" s="7">
-        <v>100.0</v>
+        <v>0.0</v>
       </c>
       <c r="C20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 3, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 4, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F20" s="4">
         <f>VLOOKUP($A20, dict!$A:$F, 6, false) * $B20 / VLOOKUP($A20, dict!$A:$F, 2, false)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -1103,7 +1103,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="7">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="C23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 3, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
@@ -1111,44 +1111,44 @@
       </c>
       <c r="D23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 4, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>20.8</v>
+        <v>15.6</v>
       </c>
       <c r="E23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 5, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>17.2</v>
+        <v>12.9</v>
       </c>
       <c r="F23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 6, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>236</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B24" s="7">
         <v>110.0</v>
       </c>
       <c r="C24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 3, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>37.4</v>
+        <v>41.8</v>
       </c>
       <c r="D24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 4, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>8.8</v>
+        <v>10.56</v>
       </c>
       <c r="E24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 5, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>2.09</v>
+        <v>1.87</v>
       </c>
       <c r="F24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 6, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>217.8</v>
+        <v>237.6</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B25" s="7">
         <v>0.0</v>
@@ -1171,10 +1171,52 @@
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="4"/>
+      <c r="A26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="C26" s="4">
+        <f>VLOOKUP($A26, dict!$A:$F, 3, false) * $B26 / VLOOKUP($A26, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="4">
+        <f>VLOOKUP($A26, dict!$A:$F, 4, false) * $B26 / VLOOKUP($A26, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <f>VLOOKUP($A26, dict!$A:$F, 5, false) * $B26 / VLOOKUP($A26, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="4">
+        <f>VLOOKUP($A26, dict!$A:$F, 6, false) * $B26 / VLOOKUP($A26, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="4"/>
+      <c r="A27" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="C27" s="4">
+        <f>VLOOKUP($A27, dict!$A:$F, 3, false) * $B27 / VLOOKUP($A27, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="4">
+        <f>VLOOKUP($A27, dict!$A:$F, 4, false) * $B27 / VLOOKUP($A27, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="4">
+        <f>VLOOKUP($A27, dict!$A:$F, 5, false) * $B27 / VLOOKUP($A27, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="4">
+        <f>VLOOKUP($A27, dict!$A:$F, 6, false) * $B27 / VLOOKUP($A27, dict!$A:$F, 2, false)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4"/>
@@ -4275,7 +4317,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
@@ -4299,7 +4341,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -7303,10 +7345,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7321,12 +7363,12 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" s="4">
         <v>1.0</v>
@@ -7346,7 +7388,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="4">
         <v>1.0</v>
@@ -7370,7 +7412,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="7">
         <v>1.0</v>
@@ -7442,7 +7484,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4">
         <v>1.0</v>
@@ -7466,7 +7508,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="7">
         <v>100.0</v>
@@ -7562,7 +7604,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="7">
         <v>100.0</v>
@@ -7586,7 +7628,7 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="4">
         <v>100.0</v>
@@ -7610,7 +7652,7 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B14" s="4">
         <v>100.0</v>
@@ -7658,7 +7700,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="7">
         <v>4.0</v>
@@ -7706,7 +7748,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7">
         <v>1.0</v>
@@ -7730,7 +7772,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="7">
         <v>1.0</v>
@@ -7754,7 +7796,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="7">
         <v>1.0</v>
@@ -7778,7 +7820,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="4">
         <v>1.0</v>
@@ -7802,7 +7844,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22" s="4">
         <v>100.0</v>
@@ -7826,7 +7868,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" s="7">
         <v>100.0</v>
@@ -7850,7 +7892,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B24" s="4">
         <v>100.0</v>
@@ -8066,7 +8108,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="B33" s="4">
         <v>100.0</v>
@@ -8090,7 +8132,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="4">
         <v>100.0</v>
@@ -8114,7 +8156,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" s="7">
         <v>100.0</v>
@@ -8138,7 +8180,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="4">
         <v>100.0</v>
@@ -8210,7 +8252,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B39" s="4">
         <v>100.0</v>
@@ -8234,7 +8276,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" s="7">
         <v>100.0</v>
@@ -8282,7 +8324,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B42" s="7">
         <v>100.0</v>
@@ -8306,7 +8348,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="B43" s="3">
         <v>100.0</v>
@@ -8354,7 +8396,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B45" s="4">
         <v>1.0</v>
@@ -8402,7 +8444,7 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47" s="4">
         <v>100.0</v>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-28
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -88,7 +88,7 @@
     <t>אורז</t>
   </si>
   <si>
-    <t xml:space="preserve">גרנולה שוקולד </t>
+    <t>קוואקר</t>
   </si>
   <si>
     <t>דבש</t>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t>אצבעות מוצרלה</t>
-  </si>
-  <si>
-    <t>קוואקר</t>
   </si>
   <si>
     <t>נודלס אורז</t>
@@ -236,6 +233,9 @@
   </si>
   <si>
     <t>פיתות כוסמין לוי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">גרנולה שוקולד </t>
   </si>
 </sst>
 </file>
@@ -595,23 +595,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>412.113</v>
+        <v>401.128</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>204.365</v>
+        <v>215.49</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>60.225</v>
+        <v>57.04</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3058.3</v>
+        <v>3015.45</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>3007.937</v>
+        <v>2979.832</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -763,23 +763,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>195.0</v>
+        <v>220.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>18.213</v>
+        <v>20.548</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>2.145</v>
+        <v>2.42</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.195</v>
+        <v>0.22</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -787,23 +787,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="5">
-        <v>300.0</v>
+        <v>270.0</v>
       </c>
       <c r="C10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>5.1</v>
+        <v>4.59</v>
       </c>
       <c r="E10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="F10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>258</v>
+        <v>232.2</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -811,7 +811,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>170.0</v>
+        <v>220.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -819,15 +819,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>42.5</v>
+        <v>55</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4.25</v>
+        <v>5.5</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>204</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -835,23 +835,23 @@
         <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="C12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 3, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>35.2</v>
+        <v>31.68</v>
       </c>
       <c r="D12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 4, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="E12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 5, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>1.3</v>
+        <v>1.17</v>
       </c>
       <c r="F12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 6, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>176.5</v>
+        <v>158.85</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -859,15 +859,15 @@
         <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="C13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 3, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>39</v>
+        <v>35.1</v>
       </c>
       <c r="D13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 4, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>4.4</v>
+        <v>3.96</v>
       </c>
       <c r="E13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 5, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
@@ -875,7 +875,7 @@
       </c>
       <c r="F13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 6, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>175</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -883,23 +883,23 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>50.0</v>
+        <v>40.0</v>
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>31.5</v>
+        <v>27.6</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>217.5</v>
+        <v>149.6</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -933,11 +933,11 @@
         <v>23</v>
       </c>
       <c r="B16" s="3">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="C16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 3, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 4, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
@@ -949,7 +949,7 @@
       </c>
       <c r="F16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 6, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -1148,7 +1148,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B25" s="7">
         <v>0.0</v>
@@ -1172,7 +1172,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" s="7">
         <v>0.0</v>
@@ -1196,7 +1196,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27" s="7">
         <v>0.0</v>
@@ -4317,7 +4317,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
@@ -4341,7 +4341,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -7345,10 +7345,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7363,12 +7363,12 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="4">
         <v>1.0</v>
@@ -7388,7 +7388,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3" s="4">
         <v>1.0</v>
@@ -7412,7 +7412,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="7">
         <v>1.0</v>
@@ -7484,7 +7484,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4">
         <v>1.0</v>
@@ -7508,7 +7508,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" s="7">
         <v>100.0</v>
@@ -7604,7 +7604,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="7">
         <v>100.0</v>
@@ -7628,7 +7628,7 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="4">
         <v>100.0</v>
@@ -7652,7 +7652,7 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4">
         <v>100.0</v>
@@ -7700,7 +7700,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="7">
         <v>4.0</v>
@@ -7748,7 +7748,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="7">
         <v>1.0</v>
@@ -7772,7 +7772,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" s="7">
         <v>1.0</v>
@@ -7796,7 +7796,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="7">
         <v>1.0</v>
@@ -7820,7 +7820,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B21" s="4">
         <v>1.0</v>
@@ -7844,7 +7844,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B22" s="4">
         <v>100.0</v>
@@ -7868,7 +7868,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" s="7">
         <v>100.0</v>
@@ -7892,7 +7892,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="4">
         <v>100.0</v>
@@ -7916,7 +7916,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4">
         <v>1.0</v>
@@ -7988,7 +7988,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B28" s="4">
         <v>1.0</v>
@@ -8036,7 +8036,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B30" s="7">
         <v>100.0</v>
@@ -8060,7 +8060,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="7">
         <v>100.0</v>
@@ -8084,7 +8084,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B32" s="7">
         <v>1.0</v>
@@ -8108,7 +8108,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" s="4">
         <v>100.0</v>
@@ -8132,7 +8132,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B34" s="4">
         <v>100.0</v>
@@ -8156,7 +8156,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B35" s="7">
         <v>100.0</v>
@@ -8180,7 +8180,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B36" s="4">
         <v>100.0</v>
@@ -8252,7 +8252,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" s="4">
         <v>100.0</v>
@@ -8276,7 +8276,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B40" s="7">
         <v>100.0</v>
@@ -8324,7 +8324,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B42" s="7">
         <v>100.0</v>
@@ -8348,7 +8348,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B43" s="3">
         <v>100.0</v>
@@ -8372,7 +8372,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B44" s="7">
         <v>100.0</v>
@@ -8396,7 +8396,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="4">
         <v>1.0</v>
@@ -8420,7 +8420,7 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B46" s="4">
         <v>100.0</v>
@@ -8444,7 +8444,7 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B47" s="4">
         <v>100.0</v>
@@ -8468,7 +8468,7 @@
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" s="7">
         <v>100.0</v>
@@ -8492,7 +8492,7 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B49" s="4">
         <v>100.0</v>
@@ -8516,7 +8516,7 @@
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B50" s="7">
         <v>100.0</v>
@@ -8540,7 +8540,7 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B51" s="4">
         <v>100.0</v>
@@ -8588,7 +8588,7 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53" s="4">
         <v>100.0</v>
@@ -8636,7 +8636,7 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B55" s="7">
         <v>1.0</v>
@@ -8660,7 +8660,7 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B56" s="7">
         <v>1.0</v>
@@ -8684,7 +8684,7 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B57" s="7">
         <v>100.0</v>
@@ -8732,7 +8732,7 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="9" t="s">
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="B59" s="7">
         <v>100.0</v>

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-03-29
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -595,23 +595,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>401.128</v>
+        <v>422.604</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>215.49</v>
+        <v>203.57</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>57.04</v>
+        <v>52.82</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3015.45</v>
+        <v>3014.95</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2979.832</v>
+        <v>2980.076</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -763,23 +763,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>220.0</v>
+        <v>260.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>20.548</v>
+        <v>24.284</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>2.42</v>
+        <v>2.86</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>88</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -787,23 +787,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="5">
-        <v>270.0</v>
+        <v>250.0</v>
       </c>
       <c r="C10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>4.59</v>
+        <v>4.25</v>
       </c>
       <c r="E10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="F10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>232.2</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -811,7 +811,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>220.0</v>
+        <v>180.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -819,15 +819,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>264</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -835,23 +835,23 @@
         <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>45.0</v>
+        <v>55.0</v>
       </c>
       <c r="C12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 3, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>31.68</v>
+        <v>38.72</v>
       </c>
       <c r="D12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 4, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="E12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 5, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>1.17</v>
+        <v>1.43</v>
       </c>
       <c r="F12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 6, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>158.85</v>
+        <v>194.15</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -859,15 +859,15 @@
         <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>45.0</v>
+        <v>55.0</v>
       </c>
       <c r="C13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 3, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>35.1</v>
+        <v>42.9</v>
       </c>
       <c r="D13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 4, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>3.96</v>
+        <v>4.84</v>
       </c>
       <c r="E13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 5, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
@@ -875,7 +875,7 @@
       </c>
       <c r="F13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 6, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>157.5</v>
+        <v>192.5</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -883,23 +883,23 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>40.0</v>
+        <v>50.0</v>
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>27.6</v>
+        <v>34.5</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4.4</v>
+        <v>5.5</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>149.6</v>
+        <v>187</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -1103,7 +1103,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="7">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="C23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 3, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
@@ -1111,15 +1111,15 @@
       </c>
       <c r="D23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 4, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>15.6</v>
+        <v>10.4</v>
       </c>
       <c r="E23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 5, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>12.9</v>
+        <v>8.6</v>
       </c>
       <c r="F23" s="4">
         <f>VLOOKUP($A23, dict!$A:$F, 6, false) * $B23 / VLOOKUP($A23, dict!$A:$F, 2, false)</f>
-        <v>177</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Auto-export snapshot for 2026-04-12
</commit_message>
<xml_diff>
--- a/macros.xlsx
+++ b/macros.xlsx
@@ -8,7 +8,7 @@
     <sheet state="visible" name="dict" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$59</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">dict!$A$1:$G$62</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="75">
   <si>
     <t>מאכל</t>
   </si>
@@ -58,7 +58,7 @@
     <t>יוגורט פרו זירו</t>
   </si>
   <si>
-    <t>פיתות כוסמין אנג'ל</t>
+    <t>פיתות כוסמין לבן</t>
   </si>
   <si>
     <t>עגלפפון</t>
@@ -82,10 +82,10 @@
     <t>חזה עוף</t>
   </si>
   <si>
-    <t>כוסמת</t>
+    <t>תערובת ירוקים</t>
   </si>
   <si>
-    <t>אורז</t>
+    <t>פסטה אוסם</t>
   </si>
   <si>
     <t>קוואקר</t>
@@ -97,7 +97,7 @@
     <t>בננה</t>
   </si>
   <si>
-    <t>יוגורט פרו מתוק</t>
+    <t>יוגורט סויה</t>
   </si>
   <si>
     <t>גיינר</t>
@@ -106,13 +106,13 @@
     <t>אצבעות מוצרלה</t>
   </si>
   <si>
-    <t>נודלס אורז</t>
-  </si>
-  <si>
     <t>טופו קשה</t>
   </si>
   <si>
-    <t>פסטרמה</t>
+    <t>טבורוג שלוש אחוז</t>
+  </si>
+  <si>
+    <t>קמח חיטה</t>
   </si>
   <si>
     <t>_</t>
@@ -133,6 +133,9 @@
     <t>אולין בוטנים קרמל</t>
   </si>
   <si>
+    <t>אורז</t>
+  </si>
+  <si>
     <t>אצבעות עמק</t>
   </si>
   <si>
@@ -148,6 +151,9 @@
     <t>גרנולה לא מתוקה</t>
   </si>
   <si>
+    <t xml:space="preserve">גרנולה שוקולד </t>
+  </si>
+  <si>
     <t>זית</t>
   </si>
   <si>
@@ -157,13 +163,13 @@
     <t>חטיף חלבון פיסטוק</t>
   </si>
   <si>
+    <t>חטיף טודיי</t>
+  </si>
+  <si>
     <t>חטיף נטור ואלי</t>
   </si>
   <si>
     <t>חלבון ביצה</t>
-  </si>
-  <si>
-    <t>טבורוג שלוש אחוז</t>
   </si>
   <si>
     <t>טונה</t>
@@ -172,7 +178,13 @@
     <t>יוגור פרו אחוז וחצי</t>
   </si>
   <si>
+    <t>יוגורט פרו מתוק</t>
+  </si>
+  <si>
     <t>כדור תמרים</t>
+  </si>
+  <si>
+    <t>כוסמת</t>
   </si>
   <si>
     <t>לחם מלא</t>
@@ -181,7 +193,13 @@
     <t>לחם שחור משרד</t>
   </si>
   <si>
+    <t>לחמנייה ברון</t>
+  </si>
+  <si>
     <t>מנה חמה בקר</t>
+  </si>
+  <si>
+    <t>נודלס אורז</t>
   </si>
   <si>
     <t>נודלס חיטה</t>
@@ -199,13 +217,16 @@
     <t>פטריות פורטבלה</t>
   </si>
   <si>
-    <t>פיתות כוסמין לבן</t>
+    <t>פיתות כוסמין אנג'ל</t>
+  </si>
+  <si>
+    <t>פיתות כוסמין לוי</t>
   </si>
   <si>
     <t>פיתות כוסמין מלא</t>
   </si>
   <si>
-    <t>פסטה אוסם</t>
+    <t>פסטרמה</t>
   </si>
   <si>
     <t>פרגית</t>
@@ -220,22 +241,10 @@
     <t>קישוא</t>
   </si>
   <si>
-    <t>קמח חיטה</t>
-  </si>
-  <si>
-    <t>תערובת ירוקים</t>
-  </si>
-  <si>
     <t>ריבר בוט בינוני</t>
   </si>
   <si>
-    <t>חטיף טודיי</t>
-  </si>
-  <si>
-    <t>פיתות כוסמין לוי</t>
-  </si>
-  <si>
-    <t xml:space="preserve">גרנולה שוקולד </t>
+    <t>מצת כוסמין</t>
   </si>
 </sst>
 </file>
@@ -595,23 +604,23 @@
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>422.604</v>
+        <v>491.48</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>203.57</v>
+        <v>228.18</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>52.82</v>
+        <v>65.34</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>3014.95</v>
+        <v>3524.2</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>2980.076</v>
+        <v>3466.7</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -619,23 +628,23 @@
         <v>12</v>
       </c>
       <c r="B3" s="3">
-        <v>110.0</v>
+        <v>150.0</v>
       </c>
       <c r="C3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 3, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>67.5</v>
       </c>
       <c r="D3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 4, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>13.95</v>
       </c>
       <c r="E3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 5, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>2.1</v>
       </c>
       <c r="F3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 6, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -715,7 +724,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="3">
-        <v>7.0</v>
+        <v>5.0</v>
       </c>
       <c r="C7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 3, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
@@ -727,11 +736,11 @@
       </c>
       <c r="E7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 5, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>6.44</v>
+        <v>4.6</v>
       </c>
       <c r="F7" s="4">
         <f>VLOOKUP($A7, dict!$A:$F, 6, false) * $B7 / VLOOKUP($A7, dict!$A:$F, 2, false)</f>
-        <v>58.1</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -763,23 +772,23 @@
         <v>17</v>
       </c>
       <c r="B9" s="3">
-        <v>260.0</v>
+        <v>200.0</v>
       </c>
       <c r="C9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 3, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>24.284</v>
+        <v>18.68</v>
       </c>
       <c r="D9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 4, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>2.86</v>
+        <v>2.2</v>
       </c>
       <c r="E9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 5, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="F9" s="4">
         <f>VLOOKUP($A9, dict!$A:$F, 6, false) * $B9 / VLOOKUP($A9, dict!$A:$F, 2, false)</f>
-        <v>104</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -787,23 +796,23 @@
         <v>18</v>
       </c>
       <c r="B10" s="5">
-        <v>250.0</v>
+        <v>0.0</v>
       </c>
       <c r="C10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 3, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 4, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 5, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F10" s="6">
         <f>VLOOKUP($A10, dict!$A:$F, 6, false) * $B10 / VLOOKUP($A10, dict!$A:$F, 2, false)</f>
-        <v>215</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -811,7 +820,7 @@
         <v>19</v>
       </c>
       <c r="B11" s="3">
-        <v>180.0</v>
+        <v>230.0</v>
       </c>
       <c r="C11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 3, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
@@ -819,15 +828,15 @@
       </c>
       <c r="D11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 4, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>45</v>
+        <v>57.5</v>
       </c>
       <c r="E11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 5, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>4.5</v>
+        <v>5.75</v>
       </c>
       <c r="F11" s="4">
         <f>VLOOKUP($A11, dict!$A:$F, 6, false) * $B11 / VLOOKUP($A11, dict!$A:$F, 2, false)</f>
-        <v>216</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -835,23 +844,23 @@
         <v>20</v>
       </c>
       <c r="B12" s="3">
-        <v>55.0</v>
+        <v>0.0</v>
       </c>
       <c r="C12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 3, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>38.72</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 4, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>6.6</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 5, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>1.43</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4">
         <f>VLOOKUP($A12, dict!$A:$F, 6, false) * $B12 / VLOOKUP($A12, dict!$A:$F, 2, false)</f>
-        <v>194.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -859,23 +868,23 @@
         <v>21</v>
       </c>
       <c r="B13" s="3">
-        <v>55.0</v>
+        <v>150.0</v>
       </c>
       <c r="C13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 3, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>42.9</v>
+        <v>106.5</v>
       </c>
       <c r="D13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 4, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>4.84</v>
+        <v>16.5</v>
       </c>
       <c r="E13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 5, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>2.25</v>
       </c>
       <c r="F13" s="4">
         <f>VLOOKUP($A13, dict!$A:$F, 6, false) * $B13 / VLOOKUP($A13, dict!$A:$F, 2, false)</f>
-        <v>192.5</v>
+        <v>523.5</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -883,23 +892,23 @@
         <v>22</v>
       </c>
       <c r="B14" s="3">
-        <v>50.0</v>
+        <v>40.0</v>
       </c>
       <c r="C14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 3, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>34.5</v>
+        <v>27.6</v>
       </c>
       <c r="D14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 4, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>5.5</v>
+        <v>4.4</v>
       </c>
       <c r="E14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 5, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F14" s="4">
         <f>VLOOKUP($A14, dict!$A:$F, 6, false) * $B14 / VLOOKUP($A14, dict!$A:$F, 2, false)</f>
-        <v>187</v>
+        <v>149.6</v>
       </c>
       <c r="G14" s="4"/>
     </row>
@@ -933,11 +942,11 @@
         <v>23</v>
       </c>
       <c r="B16" s="3">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="C16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 3, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 4, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
@@ -949,7 +958,7 @@
       </c>
       <c r="F16" s="4">
         <f>VLOOKUP($A16, dict!$A:$F, 6, false) * $B16 / VLOOKUP($A16, dict!$A:$F, 2, false)</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4"/>
     </row>
@@ -987,7 +996,7 @@
       </c>
       <c r="C18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 3, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="D18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 4, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
@@ -995,11 +1004,11 @@
       </c>
       <c r="E18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 5, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F18" s="4">
         <f>VLOOKUP($A18, dict!$A:$F, 6, false) * $B18 / VLOOKUP($A18, dict!$A:$F, 2, false)</f>
-        <v>130</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
@@ -1052,26 +1061,26 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B21" s="7">
         <v>1.0</v>
       </c>
       <c r="C21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 3, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>6.7</v>
+        <v>12</v>
       </c>
       <c r="D21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 4, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 5, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21" s="4">
         <f>VLOOKUP($A21, dict!$A:$F, 6, false) * $B21 / VLOOKUP($A21, dict!$A:$F, 2, false)</f>
-        <v>116</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -1131,48 +1140,48 @@
       </c>
       <c r="C24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 3, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>49.5</v>
       </c>
       <c r="D24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 4, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>10.23</v>
       </c>
       <c r="E24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 5, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>1.54</v>
       </c>
       <c r="F24" s="4">
         <f>VLOOKUP($A24, dict!$A:$F, 6, false) * $B24 / VLOOKUP($A24, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>259.6</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" s="7">
-        <v>0.0</v>
+        <v>100.0</v>
       </c>
       <c r="C25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 3, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="D25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 4, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 5, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F25" s="4">
         <f>VLOOKUP($A25, dict!$A:$F, 6, false) * $B25 / VLOOKUP($A25, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>349</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B26" s="7">
         <v>0.0</v>
@@ -1196,7 +1205,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="7">
         <v>0.0</v>
@@ -4201,106 +4210,106 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B2" s="3">
-        <v>110.0</v>
+        <v>250.0</v>
       </c>
       <c r="C2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 3, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>41.8</v>
+        <v>8.75</v>
       </c>
       <c r="D2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 4, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>10.56</v>
+        <v>38.5</v>
       </c>
       <c r="E2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 5, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>1.87</v>
+        <v>7.5</v>
       </c>
       <c r="F2" s="4">
         <f>VLOOKUP($A2, dict!$A:$F, 6, false) * $B2 / VLOOKUP($A2, dict!$A:$F, 2, false)</f>
-        <v>237.6</v>
+        <v>257.5</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" ref="G2:J2" si="1">SUM(C:C)</f>
-        <v>57.5</v>
+        <v>70.85</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="1"/>
-        <v>49.56</v>
+        <v>55.32</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="1"/>
-        <v>9.97</v>
+        <v>19.4</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="1"/>
-        <v>530.1</v>
+        <v>683.2</v>
       </c>
       <c r="K2" s="4">
         <f>G2*4 + H2*4 + I2*9</f>
-        <v>517.97</v>
+        <v>679.28</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="B3" s="3">
-        <v>1.0</v>
+        <v>80.0</v>
       </c>
       <c r="C3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 3, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>6.7</v>
+        <v>57.6</v>
       </c>
       <c r="D3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 4, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>21</v>
+        <v>8.32</v>
       </c>
       <c r="E3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 5, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="F3" s="4">
         <f>VLOOKUP($A3, dict!$A:$F, 6, false) * $B3 / VLOOKUP($A3, dict!$A:$F, 2, false)</f>
-        <v>116</v>
+        <v>271.2</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" s="3">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="C4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 3, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 4, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="E4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 5, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>4.6</v>
+        <v>6.5</v>
       </c>
       <c r="F4" s="4">
         <f>VLOOKUP($A4, dict!$A:$F, 6, false) * $B4 / VLOOKUP($A4, dict!$A:$F, 2, false)</f>
-        <v>41.5</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B5" s="3">
-        <v>100.0</v>
+        <v>5.0</v>
       </c>
       <c r="C5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 3, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 4, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
@@ -4308,35 +4317,35 @@
       </c>
       <c r="E5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 5, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>0</v>
+        <v>4.6</v>
       </c>
       <c r="F5" s="4">
         <f>VLOOKUP($A5, dict!$A:$F, 6, false) * $B5 / VLOOKUP($A5, dict!$A:$F, 2, false)</f>
-        <v>15</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B6" s="3">
         <v>5.0</v>
       </c>
       <c r="C6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 3, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 4, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 5, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="F6" s="4">
         <f>VLOOKUP($A6, dict!$A:$F, 6, false) * $B6 / VLOOKUP($A6, dict!$A:$F, 2, false)</f>
-        <v>120</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -7406,7 +7415,7 @@
         <v>110.0</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G59" si="1">4*C3 + 4*D3 + 9*E3</f>
+        <f t="shared" ref="G3:G62" si="1">4*C3 + 4*D3 + 9*E3</f>
         <v>113</v>
       </c>
     </row>
@@ -7436,7 +7445,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B5" s="4">
         <v>100.0</v>
@@ -7484,7 +7493,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4">
         <v>1.0</v>
@@ -7508,7 +7517,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="7">
         <v>100.0</v>
@@ -7604,7 +7613,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="7">
         <v>100.0</v>
@@ -7627,27 +7636,27 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="4">
+      <c r="A13" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="7">
         <v>100.0</v>
       </c>
-      <c r="C13" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="D13" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="E13" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="F13" s="4">
-        <v>31.0</v>
+      <c r="C13" s="7">
+        <v>72.0</v>
+      </c>
+      <c r="D13" s="7">
+        <v>16.0</v>
+      </c>
+      <c r="E13" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="F13" s="7">
+        <v>397.0</v>
       </c>
       <c r="G13" s="4">
         <f t="shared" si="1"/>
-        <v>30.7</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -7658,140 +7667,140 @@
         <v>100.0</v>
       </c>
       <c r="C14" s="4">
-        <v>51.8</v>
+        <v>6.0</v>
       </c>
       <c r="D14" s="4">
-        <v>14.7</v>
+        <v>1.0</v>
       </c>
       <c r="E14" s="4">
-        <v>14.5</v>
+        <v>0.3</v>
       </c>
       <c r="F14" s="4">
-        <v>384.0</v>
+        <v>31.0</v>
       </c>
       <c r="G14" s="4">
         <f t="shared" si="1"/>
-        <v>396.5</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="7">
+      <c r="A15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="4">
         <v>100.0</v>
       </c>
-      <c r="C15" s="7">
-        <v>80.0</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0.0</v>
-      </c>
-      <c r="E15" s="7">
-        <v>0.0</v>
-      </c>
-      <c r="F15" s="7">
-        <v>320.0</v>
+      <c r="C15" s="4">
+        <v>51.8</v>
+      </c>
+      <c r="D15" s="4">
+        <v>14.7</v>
+      </c>
+      <c r="E15" s="4">
+        <v>14.5</v>
+      </c>
+      <c r="F15" s="4">
+        <v>384.0</v>
       </c>
       <c r="G15" s="4">
         <f t="shared" si="1"/>
-        <v>320</v>
+        <v>396.5</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="7">
-        <v>4.0</v>
+        <v>100.0</v>
       </c>
       <c r="C16" s="7">
-        <v>0.0</v>
+        <v>63.0</v>
       </c>
       <c r="D16" s="7">
-        <v>0.0</v>
+        <v>9.0</v>
       </c>
       <c r="E16" s="7">
-        <v>2.0</v>
+        <v>15.0</v>
       </c>
       <c r="F16" s="7">
-        <v>15.0</v>
+        <v>435.0</v>
       </c>
       <c r="G16" s="4">
         <f t="shared" si="1"/>
-        <v>18</v>
+        <v>423</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="4">
+      <c r="A17" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="7">
         <v>100.0</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="7">
+        <v>80.0</v>
+      </c>
+      <c r="D17" s="7">
         <v>0.0</v>
       </c>
-      <c r="D17" s="4">
-        <v>25.0</v>
-      </c>
-      <c r="E17" s="4">
-        <v>2.5</v>
-      </c>
-      <c r="F17" s="4">
-        <v>120.0</v>
+      <c r="E17" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="7">
+        <v>320.0</v>
       </c>
       <c r="G17" s="4">
         <f t="shared" si="1"/>
-        <v>122.5</v>
+        <v>320</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C18" s="7">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="D18" s="7">
-        <v>21.0</v>
+        <v>0.0</v>
       </c>
       <c r="E18" s="7">
-        <v>14.0</v>
-      </c>
-      <c r="F18" s="3">
-        <v>276.0</v>
+        <v>2.0</v>
+      </c>
+      <c r="F18" s="7">
+        <v>15.0</v>
       </c>
       <c r="G18" s="4">
         <f t="shared" si="1"/>
-        <v>278</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="C19" s="7">
-        <v>21.7</v>
-      </c>
-      <c r="D19" s="7">
-        <v>15.0</v>
-      </c>
-      <c r="E19" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="F19" s="7">
-        <v>212.0</v>
+      <c r="A19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>25.0</v>
+      </c>
+      <c r="E19" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="F19" s="4">
+        <v>120.0</v>
       </c>
       <c r="G19" s="4">
         <f t="shared" si="1"/>
-        <v>236.8</v>
+        <v>122.5</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -7802,68 +7811,68 @@
         <v>1.0</v>
       </c>
       <c r="C20" s="7">
-        <v>27.0</v>
+        <v>17.0</v>
       </c>
       <c r="D20" s="7">
-        <v>3.7</v>
+        <v>21.0</v>
       </c>
       <c r="E20" s="7">
-        <v>7.5</v>
-      </c>
-      <c r="F20" s="7">
-        <v>195.0</v>
+        <v>14.0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>276.0</v>
       </c>
       <c r="G20" s="4">
         <f t="shared" si="1"/>
-        <v>190.3</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="7">
         <v>1.0</v>
       </c>
-      <c r="C21" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="D21" s="4">
-        <v>3.6</v>
-      </c>
-      <c r="E21" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="F21" s="4">
-        <v>17.2</v>
+      <c r="C21" s="7">
+        <v>21.7</v>
+      </c>
+      <c r="D21" s="7">
+        <v>15.0</v>
+      </c>
+      <c r="E21" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="F21" s="7">
+        <v>212.0</v>
       </c>
       <c r="G21" s="4">
         <f t="shared" si="1"/>
-        <v>16.1</v>
+        <v>236.8</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="4">
-        <v>100.0</v>
-      </c>
-      <c r="C22" s="4">
-        <v>3.5</v>
-      </c>
-      <c r="D22" s="4">
-        <v>15.4</v>
-      </c>
-      <c r="E22" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="F22" s="4">
-        <v>103.0</v>
+      <c r="B22" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="C22" s="7">
+        <v>16.0</v>
+      </c>
+      <c r="D22" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="E22" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="F22" s="7">
+        <v>185.0</v>
       </c>
       <c r="G22" s="4">
         <f t="shared" si="1"/>
-        <v>102.6</v>
+        <v>164.8</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -7871,892 +7880,961 @@
         <v>48</v>
       </c>
       <c r="B23" s="7">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C23" s="7">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="D23" s="7">
-        <v>24.8</v>
+        <v>3.7</v>
       </c>
       <c r="E23" s="7">
-        <v>0.6</v>
+        <v>7.5</v>
       </c>
       <c r="F23" s="7">
-        <v>104.0</v>
+        <v>195.0</v>
       </c>
       <c r="G23" s="4">
         <f t="shared" si="1"/>
-        <v>104.6</v>
+        <v>190.3</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B24" s="4">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C24" s="4">
-        <v>1.0</v>
+        <v>0.2</v>
       </c>
       <c r="D24" s="4">
-        <v>16.0</v>
+        <v>3.6</v>
       </c>
       <c r="E24" s="4">
-        <v>8.0</v>
+        <v>0.1</v>
       </c>
       <c r="F24" s="4">
-        <v>140.0</v>
+        <v>17.2</v>
       </c>
       <c r="G24" s="4">
         <f t="shared" si="1"/>
-        <v>140</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="B25" s="4">
-        <v>1.0</v>
+        <v>100.0</v>
       </c>
       <c r="C25" s="4">
-        <v>6.8</v>
+        <v>3.5</v>
       </c>
       <c r="D25" s="4">
-        <v>21.0</v>
+        <v>15.4</v>
       </c>
       <c r="E25" s="4">
         <v>3.0</v>
       </c>
       <c r="F25" s="4">
-        <v>140.0</v>
+        <v>103.0</v>
       </c>
       <c r="G25" s="4">
         <f t="shared" si="1"/>
-        <v>138.2</v>
+        <v>102.6</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B26" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="C26" s="4">
-        <v>6.7</v>
-      </c>
-      <c r="D26" s="4">
-        <v>21.0</v>
-      </c>
-      <c r="E26" s="4">
+      <c r="A26" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="7">
+        <v>100.0</v>
+      </c>
+      <c r="C26" s="7">
         <v>0.0</v>
       </c>
-      <c r="F26" s="4">
-        <v>116.0</v>
+      <c r="D26" s="7">
+        <v>24.8</v>
+      </c>
+      <c r="E26" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="F26" s="7">
+        <v>104.0</v>
       </c>
       <c r="G26" s="4">
         <f t="shared" si="1"/>
-        <v>110.8</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B27" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C27" s="4">
         <v>1.0</v>
       </c>
-      <c r="C27" s="4">
-        <v>11.2</v>
-      </c>
       <c r="D27" s="4">
-        <v>20.0</v>
+        <v>16.0</v>
       </c>
       <c r="E27" s="4">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="F27" s="4">
-        <v>130.0</v>
+        <v>140.0</v>
       </c>
       <c r="G27" s="4">
         <f t="shared" si="1"/>
-        <v>124.8</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B28" s="4">
         <v>1.0</v>
       </c>
       <c r="C28" s="4">
-        <v>15.0</v>
+        <v>6.8</v>
       </c>
       <c r="D28" s="4">
-        <v>3.0</v>
+        <v>21.0</v>
       </c>
       <c r="E28" s="4">
         <v>3.0</v>
       </c>
       <c r="F28" s="4">
-        <v>100.0</v>
+        <v>140.0</v>
       </c>
       <c r="G28" s="4">
         <f t="shared" si="1"/>
-        <v>99</v>
+        <v>138.2</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B29" s="4">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C29" s="4">
-        <v>70.4</v>
+        <v>6.7</v>
       </c>
       <c r="D29" s="4">
-        <v>12.0</v>
+        <v>21.0</v>
       </c>
       <c r="E29" s="4">
-        <v>2.6</v>
+        <v>0.0</v>
       </c>
       <c r="F29" s="4">
-        <v>353.0</v>
+        <v>116.0</v>
       </c>
       <c r="G29" s="4">
         <f t="shared" si="1"/>
-        <v>353</v>
+        <v>110.8</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="7">
-        <v>100.0</v>
-      </c>
-      <c r="C30" s="7">
-        <v>41.0</v>
-      </c>
-      <c r="D30" s="7">
-        <v>13.0</v>
-      </c>
-      <c r="E30" s="7">
-        <v>3.0</v>
-      </c>
-      <c r="F30" s="7">
-        <v>247.0</v>
+      <c r="A30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C30" s="4">
+        <v>11.2</v>
+      </c>
+      <c r="D30" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="E30" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="F30" s="4">
+        <v>130.0</v>
       </c>
       <c r="G30" s="4">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>124.8</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B31" s="7">
+      <c r="A31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C31" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="D31" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="E31" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="F31" s="4">
         <v>100.0</v>
-      </c>
-      <c r="C31" s="7">
-        <v>41.1</v>
-      </c>
-      <c r="D31" s="7">
-        <v>6.0</v>
-      </c>
-      <c r="E31" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="F31" s="7">
-        <v>207.0</v>
       </c>
       <c r="G31" s="4">
         <f t="shared" si="1"/>
-        <v>195.6</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="C32" s="7">
-        <v>45.0</v>
-      </c>
-      <c r="D32" s="7">
-        <v>7.0</v>
-      </c>
-      <c r="E32" s="7">
-        <v>13.0</v>
-      </c>
-      <c r="F32" s="7">
-        <v>325.0</v>
+      <c r="A32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C32" s="4">
+        <v>70.4</v>
+      </c>
+      <c r="D32" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="E32" s="4">
+        <v>2.6</v>
+      </c>
+      <c r="F32" s="4">
+        <v>353.0</v>
       </c>
       <c r="G32" s="4">
         <f t="shared" si="1"/>
-        <v>325</v>
+        <v>353</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" s="4">
+      <c r="A33" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="7">
         <v>100.0</v>
       </c>
-      <c r="C33" s="4">
-        <v>78.6</v>
-      </c>
-      <c r="D33" s="4">
-        <v>6.4</v>
-      </c>
-      <c r="E33" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="F33" s="4">
-        <v>351.0</v>
+      <c r="C33" s="7">
+        <v>41.0</v>
+      </c>
+      <c r="D33" s="7">
+        <v>13.0</v>
+      </c>
+      <c r="E33" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="F33" s="7">
+        <v>247.0</v>
       </c>
       <c r="G33" s="4">
         <f t="shared" si="1"/>
-        <v>347.2</v>
+        <v>243</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="4">
+      <c r="A34" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="7">
         <v>100.0</v>
       </c>
-      <c r="C34" s="4">
-        <v>78.2</v>
-      </c>
-      <c r="D34" s="4">
-        <v>11.3</v>
-      </c>
-      <c r="E34" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="F34" s="4">
-        <v>350.0</v>
+      <c r="C34" s="7">
+        <v>41.1</v>
+      </c>
+      <c r="D34" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="E34" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="F34" s="7">
+        <v>207.0</v>
       </c>
       <c r="G34" s="4">
         <f t="shared" si="1"/>
-        <v>358</v>
+        <v>195.6</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B35" s="7">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C35" s="7">
-        <v>0.0</v>
+        <v>68.0</v>
       </c>
       <c r="D35" s="7">
-        <v>17.0</v>
+        <v>10.0</v>
       </c>
       <c r="E35" s="7">
-        <v>22.0</v>
+        <v>5.0</v>
       </c>
       <c r="F35" s="7">
-        <v>274.0</v>
+        <v>360.0</v>
       </c>
       <c r="G35" s="4">
         <f t="shared" si="1"/>
-        <v>266</v>
+        <v>357</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B36" s="4">
-        <v>100.0</v>
-      </c>
-      <c r="C36" s="4">
-        <v>76.0</v>
-      </c>
-      <c r="D36" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E36" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="F36" s="4">
-        <v>304.0</v>
+      <c r="A36" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="C36" s="7">
+        <v>45.0</v>
+      </c>
+      <c r="D36" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="E36" s="7">
+        <v>13.0</v>
+      </c>
+      <c r="F36" s="7">
+        <v>325.0</v>
       </c>
       <c r="G36" s="4">
         <f t="shared" si="1"/>
-        <v>304</v>
+        <v>325</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="B37" s="4">
         <v>100.0</v>
       </c>
       <c r="C37" s="4">
-        <v>3.5</v>
+        <v>78.6</v>
       </c>
       <c r="D37" s="4">
-        <v>0.0</v>
+        <v>6.4</v>
       </c>
       <c r="E37" s="4">
-        <v>0.0</v>
+        <v>0.8</v>
       </c>
       <c r="F37" s="4">
-        <v>15.0</v>
+        <v>351.0</v>
       </c>
       <c r="G37" s="4">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>347.2</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B38" s="7">
-        <v>1.0</v>
-      </c>
-      <c r="C38" s="7">
-        <v>23.0</v>
-      </c>
-      <c r="D38" s="7">
-        <v>15.0</v>
-      </c>
-      <c r="E38" s="7">
-        <v>8.9</v>
-      </c>
-      <c r="F38" s="7">
-        <v>212.0</v>
+      <c r="A38" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C38" s="4">
+        <v>78.2</v>
+      </c>
+      <c r="D38" s="4">
+        <v>11.3</v>
+      </c>
+      <c r="E38" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="F38" s="4">
+        <v>350.0</v>
       </c>
       <c r="G38" s="4">
         <f t="shared" si="1"/>
-        <v>232.1</v>
+        <v>358</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B39" s="4">
+      <c r="A39" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" s="7">
         <v>100.0</v>
       </c>
-      <c r="C39" s="4">
-        <v>3.3</v>
-      </c>
-      <c r="D39" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="E39" s="4">
-        <v>0.3</v>
-      </c>
-      <c r="F39" s="4">
+      <c r="C39" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="D39" s="7">
+        <v>17.0</v>
+      </c>
+      <c r="E39" s="7">
         <v>22.0</v>
+      </c>
+      <c r="F39" s="7">
+        <v>274.0</v>
       </c>
       <c r="G39" s="4">
         <f t="shared" si="1"/>
-        <v>27.9</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="7">
+      <c r="A40" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="4">
         <v>100.0</v>
       </c>
-      <c r="C40" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="D40" s="7">
-        <v>2.5</v>
-      </c>
-      <c r="E40" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="F40" s="7">
-        <v>26.0</v>
+      <c r="C40" s="4">
+        <v>76.0</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E40" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="F40" s="4">
+        <v>304.0</v>
       </c>
       <c r="G40" s="4">
         <f t="shared" si="1"/>
-        <v>31.8</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B41" s="4">
         <v>100.0</v>
       </c>
       <c r="C41" s="4">
-        <v>38.0</v>
+        <v>3.5</v>
       </c>
       <c r="D41" s="4">
-        <v>9.6</v>
+        <v>0.0</v>
       </c>
       <c r="E41" s="4">
-        <v>1.7</v>
+        <v>0.0</v>
       </c>
       <c r="F41" s="4">
-        <v>216.0</v>
+        <v>15.0</v>
       </c>
       <c r="G41" s="4">
         <f t="shared" si="1"/>
-        <v>205.7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="9" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="B42" s="7">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C42" s="7">
-        <v>45.0</v>
+        <v>23.0</v>
       </c>
       <c r="D42" s="7">
-        <v>9.3</v>
+        <v>15.0</v>
       </c>
       <c r="E42" s="7">
-        <v>1.4</v>
+        <v>8.9</v>
       </c>
       <c r="F42" s="7">
-        <v>236.0</v>
+        <v>212.0</v>
       </c>
       <c r="G42" s="4">
         <f t="shared" si="1"/>
-        <v>229.8</v>
+        <v>232.1</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B43" s="3">
+      <c r="A43" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="4">
         <v>100.0</v>
       </c>
-      <c r="C43" s="3">
-        <v>34.0</v>
-      </c>
-      <c r="D43" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="E43" s="3">
-        <v>1.9</v>
-      </c>
-      <c r="F43" s="3">
-        <v>198.0</v>
+      <c r="C43" s="4">
+        <v>3.3</v>
+      </c>
+      <c r="D43" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="E43" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="F43" s="4">
+        <v>22.0</v>
       </c>
       <c r="G43" s="4">
         <f t="shared" si="1"/>
-        <v>185.1</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B44" s="7">
         <v>100.0</v>
       </c>
       <c r="C44" s="7">
-        <v>71.0</v>
+        <v>5.0</v>
       </c>
       <c r="D44" s="7">
-        <v>11.0</v>
+        <v>2.5</v>
       </c>
       <c r="E44" s="7">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="F44" s="7">
-        <v>349.0</v>
+        <v>26.0</v>
       </c>
       <c r="G44" s="4">
         <f t="shared" si="1"/>
-        <v>341.5</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="B45" s="4">
-        <v>1.0</v>
+        <v>100.0</v>
       </c>
       <c r="C45" s="4">
-        <v>1.1</v>
+        <v>38.0</v>
       </c>
       <c r="D45" s="4">
-        <v>3.6</v>
+        <v>9.6</v>
       </c>
       <c r="E45" s="4">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
       <c r="F45" s="4">
-        <v>24.0</v>
+        <v>216.0</v>
       </c>
       <c r="G45" s="4">
         <f t="shared" si="1"/>
-        <v>25.1</v>
+        <v>205.7</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B46" s="4">
+      <c r="A46" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="7">
         <v>100.0</v>
       </c>
-      <c r="C46" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D46" s="4">
-        <v>23.0</v>
-      </c>
-      <c r="E46" s="4">
-        <v>9.0</v>
-      </c>
-      <c r="F46" s="4">
-        <v>175.0</v>
+      <c r="C46" s="7">
+        <v>45.0</v>
+      </c>
+      <c r="D46" s="7">
+        <v>9.3</v>
+      </c>
+      <c r="E46" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="F46" s="7">
+        <v>236.0</v>
       </c>
       <c r="G46" s="4">
         <f t="shared" si="1"/>
-        <v>173</v>
+        <v>229.8</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B47" s="4">
+      <c r="A47" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B47" s="7">
         <v>100.0</v>
       </c>
-      <c r="C47" s="4">
-        <v>69.0</v>
-      </c>
-      <c r="D47" s="4">
-        <v>11.0</v>
-      </c>
-      <c r="E47" s="4">
-        <v>8.0</v>
-      </c>
-      <c r="F47" s="4">
-        <v>374.0</v>
+      <c r="C47" s="7">
+        <v>29.8</v>
+      </c>
+      <c r="D47" s="7">
+        <v>12.4</v>
+      </c>
+      <c r="E47" s="7">
+        <v>0.9</v>
+      </c>
+      <c r="F47" s="7">
+        <v>216.0</v>
       </c>
       <c r="G47" s="4">
         <f t="shared" si="1"/>
-        <v>392</v>
+        <v>176.9</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B48" s="7">
+      <c r="A48" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="3">
         <v>100.0</v>
       </c>
-      <c r="C48" s="7">
-        <v>1.5</v>
-      </c>
-      <c r="D48" s="7">
-        <v>11.0</v>
-      </c>
-      <c r="E48" s="7">
-        <v>5.0</v>
-      </c>
-      <c r="F48" s="7">
-        <v>95.0</v>
+      <c r="C48" s="3">
+        <v>34.0</v>
+      </c>
+      <c r="D48" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="E48" s="3">
+        <v>1.9</v>
+      </c>
+      <c r="F48" s="3">
+        <v>198.0</v>
       </c>
       <c r="G48" s="4">
         <f t="shared" si="1"/>
-        <v>95</v>
+        <v>185.1</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B49" s="4">
+      <c r="A49" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B49" s="7">
         <v>100.0</v>
       </c>
-      <c r="C49" s="4">
-        <v>16.2</v>
-      </c>
-      <c r="D49" s="4">
-        <v>9.4</v>
-      </c>
-      <c r="E49" s="4">
-        <v>0.9</v>
-      </c>
-      <c r="F49" s="4">
-        <v>133.0</v>
+      <c r="C49" s="7">
+        <v>71.0</v>
+      </c>
+      <c r="D49" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="E49" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="F49" s="7">
+        <v>349.0</v>
       </c>
       <c r="G49" s="4">
         <f t="shared" si="1"/>
-        <v>110.5</v>
+        <v>341.5</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B50" s="7">
-        <v>100.0</v>
-      </c>
-      <c r="C50" s="7">
-        <v>3.3</v>
-      </c>
-      <c r="D50" s="7">
-        <v>1.2</v>
-      </c>
-      <c r="E50" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="F50" s="7">
-        <v>16.0</v>
+      <c r="A50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B50" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C50" s="4">
+        <v>1.1</v>
+      </c>
+      <c r="D50" s="4">
+        <v>3.6</v>
+      </c>
+      <c r="E50" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="F50" s="4">
+        <v>24.0</v>
       </c>
       <c r="G50" s="4">
         <f t="shared" si="1"/>
-        <v>19.8</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B51" s="4">
         <v>100.0</v>
       </c>
       <c r="C51" s="4">
-        <v>72.0</v>
+        <v>0.0</v>
       </c>
       <c r="D51" s="4">
-        <v>10.4</v>
+        <v>23.0</v>
       </c>
       <c r="E51" s="4">
-        <v>1.0</v>
+        <v>9.0</v>
       </c>
       <c r="F51" s="4">
-        <v>339.0</v>
+        <v>175.0</v>
       </c>
       <c r="G51" s="4">
         <f t="shared" si="1"/>
-        <v>338.6</v>
+        <v>173</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B52" s="4">
         <v>100.0</v>
       </c>
       <c r="C52" s="4">
-        <v>0.0</v>
+        <v>69.0</v>
       </c>
       <c r="D52" s="4">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="E52" s="4">
-        <v>92.0</v>
+        <v>8.0</v>
       </c>
       <c r="F52" s="4">
-        <v>830.0</v>
+        <v>374.0</v>
       </c>
       <c r="G52" s="4">
         <f t="shared" si="1"/>
-        <v>828</v>
+        <v>392</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B53" s="4">
+      <c r="A53" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B53" s="7">
         <v>100.0</v>
       </c>
-      <c r="C53" s="4">
+      <c r="C53" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="D53" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="E53" s="7">
         <v>5.0</v>
       </c>
-      <c r="D53" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E53" s="4">
-        <v>0.8</v>
-      </c>
-      <c r="F53" s="4">
-        <v>50.0</v>
+      <c r="F53" s="7">
+        <v>95.0</v>
       </c>
       <c r="G53" s="4">
         <f t="shared" si="1"/>
-        <v>43.2</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="B54" s="4">
         <v>100.0</v>
       </c>
       <c r="C54" s="4">
-        <v>20.0</v>
+        <v>16.2</v>
       </c>
       <c r="D54" s="4">
-        <v>1.7</v>
+        <v>9.4</v>
       </c>
       <c r="E54" s="4">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="F54" s="4">
-        <v>86.0</v>
+        <v>133.0</v>
       </c>
       <c r="G54" s="4">
         <f t="shared" si="1"/>
-        <v>87.7</v>
+        <v>110.5</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B55" s="7">
-        <v>1.0</v>
+        <v>100.0</v>
       </c>
       <c r="C55" s="7">
-        <v>60.0</v>
+        <v>3.3</v>
       </c>
       <c r="D55" s="7">
-        <v>20.0</v>
+        <v>1.2</v>
       </c>
       <c r="E55" s="7">
-        <v>10.0</v>
+        <v>0.2</v>
       </c>
       <c r="F55" s="7">
-        <v>455.0</v>
+        <v>16.0</v>
       </c>
       <c r="G55" s="4">
         <f t="shared" si="1"/>
-        <v>410</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B56" s="7">
+      <c r="A56" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B56" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C56" s="4">
+        <v>72.0</v>
+      </c>
+      <c r="D56" s="4">
+        <v>10.4</v>
+      </c>
+      <c r="E56" s="4">
         <v>1.0</v>
       </c>
-      <c r="C56" s="7">
-        <v>16.0</v>
-      </c>
-      <c r="D56" s="7">
-        <v>18.0</v>
-      </c>
-      <c r="E56" s="7">
-        <v>3.2</v>
-      </c>
-      <c r="F56" s="7">
-        <v>185.0</v>
+      <c r="F56" s="4">
+        <v>339.0</v>
       </c>
       <c r="G56" s="4">
         <f t="shared" si="1"/>
-        <v>164.8</v>
+        <v>338.6</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B57" s="7">
-        <v>100.0</v>
+        <v>1.0</v>
       </c>
       <c r="C57" s="7">
-        <v>29.8</v>
+        <v>60.0</v>
       </c>
       <c r="D57" s="7">
-        <v>12.4</v>
+        <v>20.0</v>
       </c>
       <c r="E57" s="7">
-        <v>0.9</v>
+        <v>10.0</v>
       </c>
       <c r="F57" s="7">
-        <v>216.0</v>
+        <v>455.0</v>
       </c>
       <c r="G57" s="4">
         <f t="shared" si="1"/>
-        <v>176.9</v>
+        <v>410</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B58" s="7">
+      <c r="A58" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="4">
         <v>100.0</v>
       </c>
-      <c r="C58" s="7">
-        <v>72.0</v>
-      </c>
-      <c r="D58" s="7">
-        <v>16.0</v>
-      </c>
-      <c r="E58" s="7">
-        <v>4.0</v>
-      </c>
-      <c r="F58" s="7">
-        <v>397.0</v>
+      <c r="C58" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D58" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E58" s="4">
+        <v>92.0</v>
+      </c>
+      <c r="F58" s="4">
+        <v>830.0</v>
       </c>
       <c r="G58" s="4">
         <f t="shared" si="1"/>
-        <v>388</v>
+        <v>828</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B59" s="7">
+      <c r="A59" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="4">
         <v>100.0</v>
       </c>
-      <c r="C59" s="7">
-        <v>63.0</v>
-      </c>
-      <c r="D59" s="7">
-        <v>9.0</v>
-      </c>
-      <c r="E59" s="7">
-        <v>15.0</v>
-      </c>
-      <c r="F59" s="7">
-        <v>435.0</v>
+      <c r="C59" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="D59" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E59" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="F59" s="4">
+        <v>50.0</v>
       </c>
       <c r="G59" s="4">
         <f t="shared" si="1"/>
-        <v>423</v>
-      </c>
-    </row>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
+        <v>43.2</v>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="4">
+        <v>100.0</v>
+      </c>
+      <c r="C60" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="D60" s="4">
+        <v>1.7</v>
+      </c>
+      <c r="E60" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="F60" s="4">
+        <v>86.0</v>
+      </c>
+      <c r="G60" s="4">
+        <f t="shared" si="1"/>
+        <v>87.7</v>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B61" s="7">
+        <v>100.0</v>
+      </c>
+      <c r="C61" s="7">
+        <v>71.0</v>
+      </c>
+      <c r="D61" s="7">
+        <v>14.4</v>
+      </c>
+      <c r="E61" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="F61" s="7">
+        <v>361.0</v>
+      </c>
+      <c r="G61" s="4">
+        <f t="shared" si="1"/>
+        <v>354.2</v>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="A62" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B62" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="C62" s="7">
+        <v>12.0</v>
+      </c>
+      <c r="D62" s="7">
+        <v>20.0</v>
+      </c>
+      <c r="E62" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="F62" s="7">
+        <v>190.0</v>
+      </c>
+      <c r="G62" s="4">
+        <f t="shared" si="1"/>
+        <v>182</v>
+      </c>
+    </row>
     <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
@@ -9697,9 +9775,9 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$G$59">
-    <sortState ref="A1:G59">
-      <sortCondition ref="A1:A59"/>
+  <autoFilter ref="$A$1:$G$62">
+    <sortState ref="A1:G62">
+      <sortCondition ref="A1:A62"/>
     </sortState>
   </autoFilter>
   <drawing r:id="rId1"/>

</xml_diff>